<commit_message>
Atualiza Lista de Livros Finalizados.xlsx pelo site
</commit_message>
<xml_diff>
--- a/livros/Lista de Livros Finalizados.xlsx
+++ b/livros/Lista de Livros Finalizados.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Luiz\Desktop\Pasta Geral\0 - Antunes\Planilhas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F4485CE-6E6C-4F10-A089-DCA0EFF300FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02D6ECDE-1BE5-4308-8CE1-B86F06209956}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="786" xr2:uid="{3784A4AE-152C-4AF4-93D4-216D06209999}"/>
   </bookViews>
@@ -5530,7 +5530,7 @@
     </row>
     <row r="4" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A4" s="9">
-        <v>0</v>
+        <v>187</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>6</v>
@@ -5598,7 +5598,7 @@
     </row>
     <row r="5" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A5" s="9">
-        <v>0</v>
+        <v>186</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>6</v>

</xml_diff>